<commit_message>
add comments to activity and interaction + calculate proportion of picture with bobtail and ID + update metadata and metadata2 to correspond to 1st and 2nd session
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\stage_Curtin_Mahidol_2026\bobtail_pilot\bobtail_interactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAE97A6-4B99-4F14-BB9F-6B712E75AD9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54C5FAF6-814C-4442-A30A-E64965F1EFDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="705" yWindow="450" windowWidth="15375" windowHeight="9585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10245" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="104">
   <si>
     <t>picture</t>
   </si>
@@ -235,6 +235,120 @@
   </si>
   <si>
     <t xml:space="preserve">74	</t>
+  </si>
+  <si>
+    <t>C9_38</t>
+  </si>
+  <si>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>C9_69</t>
+  </si>
+  <si>
+    <t>C9_113</t>
+  </si>
+  <si>
+    <t>C9_115</t>
+  </si>
+  <si>
+    <t>C9_118</t>
+  </si>
+  <si>
+    <t>C9_158</t>
+  </si>
+  <si>
+    <t>C9_159</t>
+  </si>
+  <si>
+    <t>C9_160</t>
+  </si>
+  <si>
+    <t>C9_161</t>
+  </si>
+  <si>
+    <t>C9_162</t>
+  </si>
+  <si>
+    <t>C9_163</t>
+  </si>
+  <si>
+    <t>C9_164</t>
+  </si>
+  <si>
+    <t>C9_167</t>
+  </si>
+  <si>
+    <t>C9_169</t>
+  </si>
+  <si>
+    <t>C9_170</t>
+  </si>
+  <si>
+    <t>C9_194</t>
+  </si>
+  <si>
+    <t>C9_195</t>
+  </si>
+  <si>
+    <t>C9_196</t>
+  </si>
+  <si>
+    <t>C9_197</t>
+  </si>
+  <si>
+    <t>C9_198</t>
+  </si>
+  <si>
+    <t>C9_202</t>
+  </si>
+  <si>
+    <t>C9_203</t>
+  </si>
+  <si>
+    <t>C9_206</t>
+  </si>
+  <si>
+    <t>C9_212</t>
+  </si>
+  <si>
+    <t>C9_239</t>
+  </si>
+  <si>
+    <t>C9_240</t>
+  </si>
+  <si>
+    <t>C9_241</t>
+  </si>
+  <si>
+    <t>C9_242</t>
+  </si>
+  <si>
+    <t>C9_243</t>
+  </si>
+  <si>
+    <t>C9_247</t>
+  </si>
+  <si>
+    <t>C9_251</t>
+  </si>
+  <si>
+    <t>C9_254</t>
+  </si>
+  <si>
+    <t>C9_258</t>
+  </si>
+  <si>
+    <t>C9_279</t>
+  </si>
+  <si>
+    <t>C9_280</t>
+  </si>
+  <si>
+    <t>C9_295</t>
+  </si>
+  <si>
+    <t>C9_297</t>
   </si>
 </sst>
 </file>
@@ -4357,386 +4471,1477 @@
         <v>52</v>
       </c>
     </row>
-    <row r="116" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C116" s="11"/>
-    </row>
-    <row r="117" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C117" s="11"/>
-    </row>
-    <row r="118" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C118" s="11"/>
-    </row>
-    <row r="119" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C119" s="11"/>
-    </row>
-    <row r="120" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C120" s="11"/>
-    </row>
-    <row r="121" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C121" s="11"/>
-    </row>
-    <row r="122" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C122" s="11"/>
-    </row>
-    <row r="123" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C123" s="11"/>
-    </row>
-    <row r="124" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C124" s="11"/>
-    </row>
-    <row r="125" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C125" s="11"/>
-    </row>
-    <row r="126" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C126" s="11"/>
-    </row>
-    <row r="127" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C127" s="11"/>
-    </row>
-    <row r="128" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C128" s="11"/>
-    </row>
-    <row r="129" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C129" s="11"/>
-    </row>
-    <row r="130" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C130" s="11"/>
-    </row>
-    <row r="131" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C131" s="11"/>
-    </row>
-    <row r="132" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C132" s="11"/>
-    </row>
-    <row r="133" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C133" s="11"/>
-    </row>
-    <row r="134" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C134" s="11"/>
-    </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A135" s="10"/>
-      <c r="B135" s="10"/>
-      <c r="C135" s="11"/>
-      <c r="D135" s="10"/>
-      <c r="E135" s="10"/>
-      <c r="F135" s="10"/>
-      <c r="G135" s="10"/>
-      <c r="H135" s="10"/>
-      <c r="I135" s="10"/>
-      <c r="J135" s="10"/>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A136" s="10"/>
-      <c r="B136" s="10"/>
-      <c r="C136" s="11"/>
-      <c r="D136" s="10"/>
-      <c r="E136" s="10"/>
-      <c r="F136" s="10"/>
-      <c r="G136" s="10"/>
-      <c r="H136" s="10"/>
-      <c r="I136" s="10"/>
-      <c r="J136" s="10"/>
-    </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A137" s="10"/>
-      <c r="B137" s="10"/>
-      <c r="C137" s="11"/>
-      <c r="D137" s="10"/>
-      <c r="E137" s="10"/>
-      <c r="F137" s="10"/>
-      <c r="G137" s="10"/>
-      <c r="H137" s="10"/>
-      <c r="I137" s="10"/>
-      <c r="J137" s="10"/>
-    </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A138" s="10"/>
-      <c r="B138" s="10"/>
-      <c r="C138" s="11"/>
-      <c r="D138" s="10"/>
-      <c r="E138" s="10"/>
-      <c r="F138" s="10"/>
-      <c r="G138" s="10"/>
-      <c r="H138" s="10"/>
-      <c r="I138" s="10"/>
-      <c r="J138" s="10"/>
-    </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A139" s="10"/>
-      <c r="B139" s="10"/>
-      <c r="C139" s="11"/>
-      <c r="D139" s="10"/>
-      <c r="E139" s="10"/>
-      <c r="F139" s="10"/>
-      <c r="G139" s="10"/>
-      <c r="H139" s="10"/>
-      <c r="I139" s="10"/>
-      <c r="J139" s="10"/>
-    </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A140" s="10"/>
-      <c r="B140" s="10"/>
-      <c r="C140" s="11"/>
-      <c r="D140" s="10"/>
-      <c r="E140" s="10"/>
-      <c r="F140" s="10"/>
-      <c r="G140" s="10"/>
-      <c r="H140" s="10"/>
-      <c r="I140" s="10"/>
-      <c r="J140" s="10"/>
-    </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A141" s="10"/>
-      <c r="B141" s="10"/>
-      <c r="C141" s="11"/>
-      <c r="D141" s="10"/>
-      <c r="E141" s="10"/>
-      <c r="F141" s="10"/>
-      <c r="G141" s="10"/>
-      <c r="H141" s="10"/>
-      <c r="I141" s="10"/>
-      <c r="J141" s="10"/>
-    </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A142" s="10"/>
-      <c r="B142" s="10"/>
-      <c r="C142" s="11"/>
-      <c r="D142" s="10"/>
-      <c r="E142" s="10"/>
-      <c r="F142" s="10"/>
-      <c r="G142" s="10"/>
-      <c r="H142" s="10"/>
-      <c r="I142" s="10"/>
-      <c r="J142" s="10"/>
-    </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A143" s="10"/>
-      <c r="B143" s="10"/>
-      <c r="C143" s="11"/>
-      <c r="D143" s="10"/>
-      <c r="E143" s="10"/>
-      <c r="F143" s="10"/>
-      <c r="G143" s="10"/>
-      <c r="H143" s="10"/>
-      <c r="I143" s="10"/>
-      <c r="J143" s="10"/>
-    </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A144" s="10"/>
-      <c r="B144" s="10"/>
-      <c r="C144" s="11"/>
-      <c r="D144" s="10"/>
-      <c r="E144" s="10"/>
-      <c r="F144" s="10"/>
-      <c r="G144" s="10"/>
-      <c r="H144" s="10"/>
-      <c r="I144" s="10"/>
-      <c r="J144" s="10"/>
-    </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A145" s="10"/>
-      <c r="B145" s="10"/>
-      <c r="C145" s="11"/>
-      <c r="D145" s="10"/>
-      <c r="E145" s="10"/>
-      <c r="F145" s="10"/>
-      <c r="G145" s="10"/>
-      <c r="H145" s="10"/>
-      <c r="I145" s="10"/>
-      <c r="J145" s="10"/>
-    </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A146" s="10"/>
-      <c r="B146" s="10"/>
-      <c r="C146" s="11"/>
-      <c r="D146" s="10"/>
-      <c r="E146" s="10"/>
-      <c r="F146" s="10"/>
-      <c r="G146" s="10"/>
-      <c r="H146" s="10"/>
-      <c r="I146" s="10"/>
-      <c r="J146" s="10"/>
-    </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A147" s="10"/>
-      <c r="B147" s="10"/>
-      <c r="C147" s="11"/>
-      <c r="D147" s="10"/>
-      <c r="E147" s="10"/>
-      <c r="F147" s="10"/>
-      <c r="G147" s="10"/>
-      <c r="H147" s="10"/>
-      <c r="I147" s="10"/>
-      <c r="J147" s="10"/>
-    </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A148" s="10"/>
-      <c r="B148" s="10"/>
-      <c r="C148" s="11"/>
-      <c r="D148" s="10"/>
-      <c r="E148" s="10"/>
-      <c r="F148" s="10"/>
-      <c r="G148" s="10"/>
-      <c r="H148" s="10"/>
-      <c r="I148" s="10"/>
-      <c r="J148" s="10"/>
-    </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A149" s="10"/>
-      <c r="B149" s="10"/>
-      <c r="C149" s="11"/>
-      <c r="D149" s="10"/>
-      <c r="E149" s="10"/>
-      <c r="F149" s="10"/>
-      <c r="G149" s="10"/>
-      <c r="H149" s="10"/>
-      <c r="I149" s="10"/>
-      <c r="J149" s="10"/>
-    </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A150" s="10"/>
-      <c r="B150" s="10"/>
-      <c r="C150" s="11"/>
-      <c r="D150" s="10"/>
-      <c r="E150" s="10"/>
-      <c r="F150" s="10"/>
-      <c r="G150" s="10"/>
-      <c r="H150" s="10"/>
-      <c r="I150" s="10"/>
-      <c r="J150" s="10"/>
-    </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A151" s="10"/>
-      <c r="B151" s="10"/>
-      <c r="C151" s="11"/>
-      <c r="D151" s="10"/>
-      <c r="E151" s="10"/>
-      <c r="F151" s="10"/>
-      <c r="G151" s="10"/>
-      <c r="H151" s="10"/>
-      <c r="I151" s="10"/>
-      <c r="J151" s="10"/>
-    </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A152" s="10"/>
-      <c r="B152" s="10"/>
-      <c r="C152" s="11"/>
-      <c r="D152" s="10"/>
-      <c r="E152" s="10"/>
-      <c r="F152" s="10"/>
-      <c r="G152" s="10"/>
-      <c r="H152" s="10"/>
-      <c r="I152" s="10"/>
-      <c r="J152" s="10"/>
-    </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A153" s="10"/>
-      <c r="B153" s="10"/>
-      <c r="C153" s="11"/>
-      <c r="D153" s="10"/>
-      <c r="E153" s="10"/>
-      <c r="F153" s="10"/>
-      <c r="G153" s="10"/>
-      <c r="H153" s="10"/>
-      <c r="I153" s="10"/>
-      <c r="J153" s="10"/>
-    </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A154" s="10"/>
-      <c r="B154" s="10"/>
-      <c r="C154" s="11"/>
-      <c r="D154" s="10"/>
-      <c r="E154" s="10"/>
-      <c r="F154" s="10"/>
-      <c r="G154" s="10"/>
-      <c r="H154" s="10"/>
-      <c r="I154" s="10"/>
-      <c r="J154" s="10"/>
-    </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A155" s="10"/>
-      <c r="B155" s="10"/>
-      <c r="C155" s="11"/>
-      <c r="D155" s="10"/>
-      <c r="E155" s="10"/>
-      <c r="F155" s="10"/>
-      <c r="G155" s="10"/>
-      <c r="H155" s="10"/>
-      <c r="I155" s="10"/>
-      <c r="J155" s="10"/>
-    </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A156" s="10"/>
-      <c r="B156" s="10"/>
-      <c r="C156" s="11"/>
-      <c r="D156" s="10"/>
-      <c r="E156" s="10"/>
-      <c r="F156" s="10"/>
-      <c r="G156" s="10"/>
-      <c r="H156" s="10"/>
-      <c r="I156" s="10"/>
-      <c r="J156" s="10"/>
-    </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A157" s="10"/>
-      <c r="B157" s="10"/>
-      <c r="C157" s="11"/>
-      <c r="D157" s="10"/>
-      <c r="E157" s="10"/>
-      <c r="F157" s="10"/>
-      <c r="G157" s="10"/>
-      <c r="H157" s="10"/>
-      <c r="I157" s="10"/>
-      <c r="J157" s="10"/>
-    </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A158" s="10"/>
-      <c r="B158" s="10"/>
-      <c r="C158" s="11"/>
-      <c r="D158" s="10"/>
-      <c r="E158" s="10"/>
-      <c r="F158" s="10"/>
-      <c r="G158" s="10"/>
-      <c r="H158" s="10"/>
-      <c r="I158" s="10"/>
-      <c r="J158" s="10"/>
-    </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A159" s="10"/>
-      <c r="B159" s="10"/>
-      <c r="C159" s="11"/>
-      <c r="D159" s="10"/>
-      <c r="E159" s="10"/>
-      <c r="F159" s="10"/>
-      <c r="G159" s="10"/>
-      <c r="H159" s="10"/>
-      <c r="I159" s="10"/>
-      <c r="J159" s="10"/>
-    </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A160" s="10"/>
-      <c r="B160" s="10"/>
-      <c r="C160" s="11"/>
-      <c r="D160" s="10"/>
-      <c r="E160" s="10"/>
-      <c r="F160" s="10"/>
-      <c r="G160" s="10"/>
-      <c r="H160" s="10"/>
-      <c r="I160" s="10"/>
-      <c r="J160" s="10"/>
-    </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A161" s="10"/>
-      <c r="B161" s="10"/>
-      <c r="C161" s="11"/>
-      <c r="D161" s="10"/>
-      <c r="E161" s="10"/>
-      <c r="F161" s="10"/>
-      <c r="G161" s="10"/>
-      <c r="H161" s="10"/>
-      <c r="I161" s="10"/>
-      <c r="J161" s="10"/>
+    <row r="116" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B116" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C116" s="13">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="D116" s="12">
+        <v>1</v>
+      </c>
+      <c r="E116" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F116" s="12">
+        <v>39</v>
+      </c>
+      <c r="G116" s="14">
+        <v>20.3</v>
+      </c>
+      <c r="H116" s="14">
+        <v>27.4</v>
+      </c>
+      <c r="I116" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J116" s="14">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A117" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B117" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C117" s="13">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="D117" s="12">
+        <v>7</v>
+      </c>
+      <c r="E117" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F117" s="12">
+        <v>26</v>
+      </c>
+      <c r="G117" s="16">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="H117" s="16">
+        <v>21</v>
+      </c>
+      <c r="I117" s="16">
+        <v>74</v>
+      </c>
+      <c r="J117" s="16">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A118" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B118" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C118" s="13">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="D118" s="12">
+        <v>8</v>
+      </c>
+      <c r="E118" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F118" s="12">
+        <v>26</v>
+      </c>
+      <c r="G118" s="12">
+        <v>14.9</v>
+      </c>
+      <c r="H118" s="16">
+        <v>19.5</v>
+      </c>
+      <c r="I118" s="16">
+        <v>74</v>
+      </c>
+      <c r="J118" s="16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A119" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B119" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C119" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="D119" s="12">
+        <v>3</v>
+      </c>
+      <c r="E119" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F119" s="12">
+        <v>28</v>
+      </c>
+      <c r="G119" s="12">
+        <v>14.9</v>
+      </c>
+      <c r="H119" s="16">
+        <v>19.5</v>
+      </c>
+      <c r="I119" s="16">
+        <v>74</v>
+      </c>
+      <c r="J119" s="16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A120" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B120" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C120" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="D120" s="12">
+        <v>4</v>
+      </c>
+      <c r="E120" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F120" s="12">
+        <v>28</v>
+      </c>
+      <c r="G120" s="12">
+        <v>14.9</v>
+      </c>
+      <c r="H120" s="16">
+        <v>19.5</v>
+      </c>
+      <c r="I120" s="16">
+        <v>74</v>
+      </c>
+      <c r="J120" s="16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A121" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B121" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C121" s="13">
+        <v>0.53125</v>
+      </c>
+      <c r="D121" s="12">
+        <v>4</v>
+      </c>
+      <c r="E121" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F121" s="12">
+        <v>30</v>
+      </c>
+      <c r="G121" s="12">
+        <v>14.9</v>
+      </c>
+      <c r="H121" s="16">
+        <v>19.5</v>
+      </c>
+      <c r="I121" s="16">
+        <v>74</v>
+      </c>
+      <c r="J121" s="16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A122" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B122" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C122" s="13">
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="D122" s="12">
+        <v>7</v>
+      </c>
+      <c r="E122" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F122" s="12">
+        <v>28</v>
+      </c>
+      <c r="G122" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H122" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I122" s="14">
+        <v>63</v>
+      </c>
+      <c r="J122" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B123" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C123" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="D123" s="12">
+        <v>1</v>
+      </c>
+      <c r="E123" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F123" s="12">
+        <v>29</v>
+      </c>
+      <c r="G123" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H123" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I123" s="14">
+        <v>63</v>
+      </c>
+      <c r="J123" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B124" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C124" s="13">
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="D124" s="12">
+        <v>5</v>
+      </c>
+      <c r="E124" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F124" s="12">
+        <v>31</v>
+      </c>
+      <c r="G124" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H124" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I124" s="14">
+        <v>63</v>
+      </c>
+      <c r="J124" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A125" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B125" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C125" s="13">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="D125" s="12">
+        <v>7</v>
+      </c>
+      <c r="E125" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F125" s="12">
+        <v>30</v>
+      </c>
+      <c r="G125" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H125" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I125" s="14">
+        <v>63</v>
+      </c>
+      <c r="J125" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A126" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B126" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C126" s="13">
+        <v>0.53125</v>
+      </c>
+      <c r="D126" s="12">
+        <v>2</v>
+      </c>
+      <c r="E126" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F126" s="12">
+        <v>30</v>
+      </c>
+      <c r="G126" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H126" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I126" s="14">
+        <v>63</v>
+      </c>
+      <c r="J126" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A127" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B127" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C127" s="13">
+        <v>0.53125</v>
+      </c>
+      <c r="D127" s="12">
+        <v>8</v>
+      </c>
+      <c r="E127" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F127" s="12">
+        <v>30</v>
+      </c>
+      <c r="G127" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H127" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I127" s="14">
+        <v>63</v>
+      </c>
+      <c r="J127" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A128" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B128" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C128" s="13">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="D128" s="12">
+        <v>8</v>
+      </c>
+      <c r="E128" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F128" s="12">
+        <v>31</v>
+      </c>
+      <c r="G128" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H128" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I128" s="14">
+        <v>63</v>
+      </c>
+      <c r="J128" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A129" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B129" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C129" s="13">
+        <v>0.55208333333333304</v>
+      </c>
+      <c r="D129" s="12">
+        <v>6</v>
+      </c>
+      <c r="E129" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F129" s="12">
+        <v>32</v>
+      </c>
+      <c r="G129" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H129" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I129" s="14">
+        <v>63</v>
+      </c>
+      <c r="J129" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A130" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B130" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C130" s="13">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D130" s="12">
+        <v>1</v>
+      </c>
+      <c r="E130" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F130" s="12">
+        <v>31</v>
+      </c>
+      <c r="G130" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H130" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I130" s="14">
+        <v>63</v>
+      </c>
+      <c r="J130" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A131" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B131" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C131" s="13">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D131" s="12">
+        <v>1</v>
+      </c>
+      <c r="E131" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F131" s="12">
+        <v>33</v>
+      </c>
+      <c r="G131" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H131" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I131" s="14">
+        <v>63</v>
+      </c>
+      <c r="J131" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A132" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B132" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C132" s="13">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="D132" s="12">
+        <v>1</v>
+      </c>
+      <c r="E132" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F132" s="12">
+        <v>33</v>
+      </c>
+      <c r="G132" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="H132" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="I132" s="14">
+        <v>63</v>
+      </c>
+      <c r="J132" s="14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A133" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B133" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C133" s="13">
+        <v>0.40625</v>
+      </c>
+      <c r="D133" s="12">
+        <v>7</v>
+      </c>
+      <c r="E133" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F133" s="12">
+        <v>18</v>
+      </c>
+      <c r="G133" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H133" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I133" s="15">
+        <v>60</v>
+      </c>
+      <c r="J133" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B134" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C134" s="13">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D134" s="12">
+        <v>1</v>
+      </c>
+      <c r="E134" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F134" s="12">
+        <v>19</v>
+      </c>
+      <c r="G134" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H134" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I134" s="15">
+        <v>60</v>
+      </c>
+      <c r="J134" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B135" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C135" s="13">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D135" s="12">
+        <v>7</v>
+      </c>
+      <c r="E135" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F135" s="12">
+        <v>19</v>
+      </c>
+      <c r="G135" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H135" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I135" s="15">
+        <v>60</v>
+      </c>
+      <c r="J135" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B136" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C136" s="13">
+        <v>0.42708333333333298</v>
+      </c>
+      <c r="D136" s="12">
+        <v>1</v>
+      </c>
+      <c r="E136" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F136" s="12">
+        <v>20</v>
+      </c>
+      <c r="G136" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H136" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I136" s="15">
+        <v>60</v>
+      </c>
+      <c r="J136" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A137" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B137" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C137" s="13">
+        <v>0.42708333333333298</v>
+      </c>
+      <c r="D137" s="12">
+        <v>7</v>
+      </c>
+      <c r="E137" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F137" s="12">
+        <v>20</v>
+      </c>
+      <c r="G137" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H137" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I137" s="15">
+        <v>60</v>
+      </c>
+      <c r="J137" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A138" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B138" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C138" s="13">
+        <v>0.4375</v>
+      </c>
+      <c r="D138" s="12">
+        <v>1</v>
+      </c>
+      <c r="E138" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F138" s="12">
+        <v>21</v>
+      </c>
+      <c r="G138" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H138" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I138" s="15">
+        <v>60</v>
+      </c>
+      <c r="J138" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A139" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B139" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C139" s="13">
+        <v>0.4375</v>
+      </c>
+      <c r="D139" s="12">
+        <v>7</v>
+      </c>
+      <c r="E139" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F139" s="12">
+        <v>21</v>
+      </c>
+      <c r="G139" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H139" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I139" s="15">
+        <v>60</v>
+      </c>
+      <c r="J139" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A140" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B140" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C140" s="13">
+        <v>0.44791666666666702</v>
+      </c>
+      <c r="D140" s="12">
+        <v>1</v>
+      </c>
+      <c r="E140" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F140" s="12">
+        <v>24</v>
+      </c>
+      <c r="G140" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H140" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I140" s="15">
+        <v>60</v>
+      </c>
+      <c r="J140" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A141" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="B141" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C141" s="13">
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="D141" s="12">
+        <v>8</v>
+      </c>
+      <c r="E141" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F141" s="12">
+        <v>32</v>
+      </c>
+      <c r="G141" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H141" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I141" s="15">
+        <v>60</v>
+      </c>
+      <c r="J141" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A142" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="B142" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C142" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="D142" s="12">
+        <v>4</v>
+      </c>
+      <c r="E142" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F142" s="12">
+        <v>33</v>
+      </c>
+      <c r="G142" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H142" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I142" s="15">
+        <v>60</v>
+      </c>
+      <c r="J142" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A143" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B143" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C143" s="13">
+        <v>0.53125</v>
+      </c>
+      <c r="D143" s="12">
+        <v>4</v>
+      </c>
+      <c r="E143" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F143" s="12">
+        <v>35</v>
+      </c>
+      <c r="G143" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H143" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I143" s="15">
+        <v>60</v>
+      </c>
+      <c r="J143" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A144" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="B144" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C144" s="13">
+        <v>0.59375</v>
+      </c>
+      <c r="D144" s="12">
+        <v>4</v>
+      </c>
+      <c r="E144" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F144" s="12">
+        <v>30</v>
+      </c>
+      <c r="G144" s="14">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="H144" s="14">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="I144" s="15">
+        <v>60</v>
+      </c>
+      <c r="J144" s="15">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A145" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B145" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C145" s="13">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="D145" s="12">
+        <v>4</v>
+      </c>
+      <c r="E145" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F145" s="12">
+        <v>15</v>
+      </c>
+      <c r="G145" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H145" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I145" s="15">
+        <v>69</v>
+      </c>
+      <c r="J145" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A146" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B146" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C146" s="13">
+        <v>0.4375</v>
+      </c>
+      <c r="D146" s="12">
+        <v>2</v>
+      </c>
+      <c r="E146" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F146" s="12">
+        <v>16</v>
+      </c>
+      <c r="G146" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H146" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I146" s="15">
+        <v>69</v>
+      </c>
+      <c r="J146" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A147" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B147" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C147" s="13">
+        <v>0.4375</v>
+      </c>
+      <c r="D147" s="12">
+        <v>4</v>
+      </c>
+      <c r="E147" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F147" s="12">
+        <v>16</v>
+      </c>
+      <c r="G147" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H147" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I147" s="15">
+        <v>69</v>
+      </c>
+      <c r="J147" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A148" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B148" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C148" s="13">
+        <v>0.44791666666666702</v>
+      </c>
+      <c r="D148" s="12">
+        <v>2</v>
+      </c>
+      <c r="E148" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F148" s="12">
+        <v>19</v>
+      </c>
+      <c r="G148" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H148" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I148" s="15">
+        <v>69</v>
+      </c>
+      <c r="J148" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="149" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A149" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B149" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C149" s="13">
+        <v>0.44791666666666702</v>
+      </c>
+      <c r="D149" s="12">
+        <v>4</v>
+      </c>
+      <c r="E149" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F149" s="12">
+        <v>19</v>
+      </c>
+      <c r="G149" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H149" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I149" s="15">
+        <v>69</v>
+      </c>
+      <c r="J149" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="150" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A150" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B150" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C150" s="13">
+        <v>0.45833333333333298</v>
+      </c>
+      <c r="D150" s="12">
+        <v>4</v>
+      </c>
+      <c r="E150" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F150" s="12">
+        <v>21</v>
+      </c>
+      <c r="G150" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H150" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I150" s="15">
+        <v>69</v>
+      </c>
+      <c r="J150" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A151" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="B151" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C151" s="13">
+        <v>0.46875</v>
+      </c>
+      <c r="D151" s="12">
+        <v>1</v>
+      </c>
+      <c r="E151" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F151" s="12">
+        <v>20</v>
+      </c>
+      <c r="G151" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H151" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I151" s="15">
+        <v>69</v>
+      </c>
+      <c r="J151" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A152" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B152" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C152" s="13">
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="D152" s="12">
+        <v>3</v>
+      </c>
+      <c r="E152" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F152" s="12">
+        <v>23</v>
+      </c>
+      <c r="G152" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H152" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I152" s="15">
+        <v>69</v>
+      </c>
+      <c r="J152" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A153" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B153" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C153" s="13">
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="D153" s="12">
+        <v>5</v>
+      </c>
+      <c r="E153" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F153" s="12">
+        <v>23</v>
+      </c>
+      <c r="G153" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H153" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I153" s="15">
+        <v>69</v>
+      </c>
+      <c r="J153" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A154" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="B154" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C154" s="13">
+        <v>0.55208333333333337</v>
+      </c>
+      <c r="D154" s="12">
+        <v>4</v>
+      </c>
+      <c r="E154" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F154" s="12">
+        <v>29</v>
+      </c>
+      <c r="G154" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H154" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I154" s="15">
+        <v>69</v>
+      </c>
+      <c r="J154" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A155" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="B155" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C155" s="13">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D155" s="12">
+        <v>8</v>
+      </c>
+      <c r="E155" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F155" s="12">
+        <v>29</v>
+      </c>
+      <c r="G155" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H155" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I155" s="15">
+        <v>69</v>
+      </c>
+      <c r="J155" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A156" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B156" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C156" s="13">
+        <v>0.625</v>
+      </c>
+      <c r="D156" s="12">
+        <v>4</v>
+      </c>
+      <c r="E156" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F156" s="12">
+        <v>30</v>
+      </c>
+      <c r="G156" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H156" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I156" s="15">
+        <v>69</v>
+      </c>
+      <c r="J156" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A157" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B157" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C157" s="13">
+        <v>0.625</v>
+      </c>
+      <c r="D157" s="12">
+        <v>7</v>
+      </c>
+      <c r="E157" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F157" s="12">
+        <v>30</v>
+      </c>
+      <c r="G157" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="H157" s="14">
+        <v>16.8</v>
+      </c>
+      <c r="I157" s="15">
+        <v>69</v>
+      </c>
+      <c r="J157" s="15">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A158" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="B158" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C158" s="13">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="D158" s="12">
+        <v>4</v>
+      </c>
+      <c r="E158" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F158" s="12">
+        <v>13</v>
+      </c>
+      <c r="G158" s="16">
+        <v>14.2</v>
+      </c>
+      <c r="H158" s="14">
+        <v>21.8</v>
+      </c>
+      <c r="I158" s="15">
+        <v>56</v>
+      </c>
+      <c r="J158" s="15">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="159" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A159" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="B159" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C159" s="13">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="D159" s="12">
+        <v>6</v>
+      </c>
+      <c r="E159" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F159" s="12">
+        <v>14</v>
+      </c>
+      <c r="G159" s="16">
+        <v>14.2</v>
+      </c>
+      <c r="H159" s="14">
+        <v>21.8</v>
+      </c>
+      <c r="I159" s="15">
+        <v>56</v>
+      </c>
+      <c r="J159" s="15">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A160" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="B160" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C160" s="13">
+        <v>0.55208333333333337</v>
+      </c>
+      <c r="D160" s="12">
+        <v>4</v>
+      </c>
+      <c r="E160" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F160" s="12">
+        <v>35</v>
+      </c>
+      <c r="G160" s="16">
+        <v>14.2</v>
+      </c>
+      <c r="H160" s="14">
+        <v>21.8</v>
+      </c>
+      <c r="I160" s="15">
+        <v>56</v>
+      </c>
+      <c r="J160" s="15">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="161" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A161" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="B161" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C161" s="13">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="D161" s="12">
+        <v>5</v>
+      </c>
+      <c r="E161" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F161" s="12">
+        <v>36</v>
+      </c>
+      <c r="G161" s="16">
+        <v>14.2</v>
+      </c>
+      <c r="H161" s="14">
+        <v>21.8</v>
+      </c>
+      <c r="I161" s="15">
+        <v>56</v>
+      </c>
+      <c r="J161" s="15">
+        <v>34</v>
+      </c>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162" s="10"/>

</xml_diff>